<commit_message>
Sikring 3 A fladsikring i stedet for 3,15 A træg
3,15 A træg findes kun som 5 × 20 mm glassikring. 3 A ATO (Littelfuse
0287003.PXCN) passer i den nuværende holder og er under grænsen på
4,16 A. Ledningsdiagram v8, teknisk fil, kravoversigt og produktionslog
rettet; WLED-strømloft 2000 mA i diagrammet.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019HVS75R63EMcd4SGuc8ssb
</commit_message>
<xml_diff>
--- a/hardware/dokumentation/halo-gen2-v8_produktionslog.xlsx
+++ b/hardware/dokumentation/halo-gen2-v8_produktionslog.xlsx
@@ -460,6 +460,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -493,7 +494,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Sikring 3,15 A ✔</t>
+          <t>Sikring 3 A ✔</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -628,7 +629,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Sikring 3,15 A træg sidder i holderen på 24 V-plus</t>
+          <t>Sikring 3 A (fladsikring, violet) sidder i holderen på 24 V-plus</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr"/>
@@ -809,6 +810,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Sikring 3 A fladsikring i stedet for 3,15 A træg (#61)
3,15 A træg findes kun som 5 × 20 mm glassikring. 3 A ATO (Littelfuse
0287003.PXCN) passer i den nuværende holder og er under grænsen på
4,16 A. Ledningsdiagram v8, teknisk fil, kravoversigt og produktionslog
rettet; WLED-strømloft 2000 mA i diagrammet.


Claude-Session: https://claude.ai/code/session_019HVS75R63EMcd4SGuc8ssb

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hardware/dokumentation/halo-gen2-v8_produktionslog.xlsx
+++ b/hardware/dokumentation/halo-gen2-v8_produktionslog.xlsx
@@ -460,6 +460,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -493,7 +494,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Sikring 3,15 A ✔</t>
+          <t>Sikring 3 A ✔</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -628,7 +629,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Sikring 3,15 A træg sidder i holderen på 24 V-plus</t>
+          <t>Sikring 3 A (fladsikring, violet) sidder i holderen på 24 V-plus</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr"/>
@@ -809,6 +810,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>

</xml_diff>